<commit_message>
UPD : Further refining unit test
</commit_message>
<xml_diff>
--- a/inst/extdata/IQRtoolsExampleProject/PKModelCovariance.xlsx
+++ b/inst/extdata/IQRtoolsExampleProject/PKModelCovariance.xlsx
@@ -1152,7 +1152,7 @@
         <v>0.0029268</v>
       </c>
       <c r="F10">
-        <v>-9.3782e-05</v>
+        <v>-9.3782E-05</v>
       </c>
       <c r="G10">
         <v>0</v>
@@ -1223,7 +1223,7 @@
         <v>-0.009982100000000001</v>
       </c>
       <c r="F12">
-        <v>6.3525e-05</v>
+        <v>6.3525E-05</v>
       </c>
       <c r="G12">
         <v>0</v>

</xml_diff>